<commit_message>
change sheet name from pt-br to original
</commit_message>
<xml_diff>
--- a/data/codebook/Q12.xlsx
+++ b/data/codebook/Q12.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PT-BR" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Original" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EN-US" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
@@ -569,7 +569,7 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="19" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>RQ1</t>
         </is>
@@ -581,7 +581,7 @@
       <c r="F1" s="21" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="22" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>Q12: For those characteristics that you considered important, please describe the reason for your rating. (Optional)</t>
         </is>
@@ -601,55 +601,55 @@
       <c r="F3" s="27" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>Sub categoria</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="31" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
+      <c r="D4" s="32" t="inlineStr">
         <is>
           <t>Quote</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E4" s="33" t="inlineStr">
         <is>
           <t>Resposta</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="34" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="35" t="inlineStr">
         <is>
           <t>QUALIDADE DOS DADOS COMO FUNDAMENTO INEGOCIÁVEL</t>
         </is>
       </c>
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="35" t="inlineStr">
         <is>
           <t>Princípio "Garbage In, Garbage Out"</t>
         </is>
       </c>
       <c r="C5" s="16" t="n"/>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="35" t="inlineStr">
         <is>
           <t>If the data is a mess, the model will only produce sophisticated garbage.</t>
         </is>
       </c>
-      <c r="E5" s="17" t="inlineStr">
+      <c r="E5" s="36" t="inlineStr">
         <is>
           <t>If the data is a mess, the model will only produce sophisticated garbage.</t>
         </is>
@@ -661,23 +661,23 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="35" t="inlineStr">
         <is>
           <t>HIERARQUIZAÇÃO E RELATIVIZAÇÃO DA IMPORTÂNCIA</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B6" s="35" t="inlineStr">
         <is>
           <t>Distinção entre "fundamental no início" vs. "corrigível no processo</t>
         </is>
       </c>
       <c r="C6" s="16" t="n"/>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="35" t="inlineStr">
         <is>
           <t>Documentation issues, making this data accessible and consistent across different databases, can be corrected during the process, although they are also very important.</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="37" t="inlineStr">
         <is>
           <t>All characteristics are either important or very important. The separation I made was more about considering something we can do/correct later or something that is fundamental to consider from the beginning. I believe that anything that reflects on the quality of the data, the information present in that data, is non-negotiable from the initial moment. Documentation issues, making this data accessible and consistent across different databases, can be corrected during the process, although they are also very important.</t>
         </is>
@@ -689,23 +689,23 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="35" t="inlineStr">
         <is>
           <t>QUALIDADE DOS DADOS COMO FUNDAMENTO INEGOCIÁVEL</t>
         </is>
       </c>
-      <c r="B7" s="15" t="inlineStr">
+      <c r="B7" s="35" t="inlineStr">
         <is>
           <t>Caráter não-negociável da qualidade desde o início</t>
         </is>
       </c>
       <c r="C7" s="16" t="n"/>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="35" t="inlineStr">
         <is>
           <t>"I believe that anything that reflects on the quality of the data, the information present in that data, is non-negotiable from the initial moment.", “Poor quality data (and here poor quality ranges from lack of availability to data with low precision and low representativeness) is a major problem in the field and hinders the development of new techniques.”</t>
         </is>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="37" t="inlineStr">
         <is>
           <t>All characteristics are either important or very important. The separation I made was more about considering something we can do/correct later or something that is fundamental to consider from the beginning. I believe that anything that reflects on the quality of the data, the information present in that data, is non-negotiable from the initial moment. Documentation issues, making this data accessible and consistent across different databases, can be corrected during the process, although they are also very important.</t>
         </is>
@@ -717,23 +717,23 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>QUALIDADE DOS DADOS COMO FUNDAMENTO INEGOCIÁVEL</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B8" s="35" t="inlineStr">
         <is>
           <t>Impacto positivo no desenvolvimento de sistemas de ML</t>
         </is>
       </c>
       <c r="C8" s="16" t="n"/>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="35" t="inlineStr">
         <is>
           <t>“all these characteristics are extremely important, as guaranteeing them very positively influences the development of systems that use machine learning.”, “Poor quality data (and here poor quality ranges from lack of availability to data with low precision and low representativeness) is a major problem in the field and hinders the development of new techniques.”</t>
         </is>
       </c>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="E8" s="37" t="inlineStr">
         <is>
           <t>For me, all these characteristics are extremely important, as guaranteeing them very positively influences the development of systems that use machine learning. Poor quality data (and here poor quality ranges from lack of availability to data with low precision and low representativeness) is a major problem in the field and hinders the development of new techniques.</t>
         </is>
@@ -745,23 +745,23 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="35" t="inlineStr">
         <is>
           <t>Precisão como atributo fundamental</t>
         </is>
       </c>
       <c r="C9" s="16" t="n"/>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="35" t="inlineStr">
         <is>
           <t>“Data precision should reflect efficiently and without errors, to which it is proposed or indicated.”, “The data needs to be understandable to humans to a certain extent.”, “It needs to be reliable, in terms of ensuring that the final information is not wrong when compared to what is expected in the real world.” ,</t>
         </is>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="36" t="inlineStr">
         <is>
           <t>Data precision should reflect efficiently and without errors, to which it is proposed or indicated; the data needs to be understandable to humans to a certain extent, and it needs to be reliable, in terms of ensuring that the final information is not wrong when compared to what is expected in the real world.</t>
         </is>
@@ -773,23 +773,23 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="35" t="inlineStr">
         <is>
           <t>DEPENDÊNCIA CONTEXTUAL</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B10" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve"> Dependência do escopo do projeto</t>
         </is>
       </c>
       <c r="C10" s="16" t="n"/>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="35" t="inlineStr">
         <is>
           <t>They depend on the scope of the project and the learning objective.</t>
         </is>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E10" s="36" t="inlineStr">
         <is>
           <t>They depend on the scope of the project and the learning objective.</t>
         </is>
@@ -801,23 +801,23 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B11" s="15" t="inlineStr">
+      <c r="B11" s="35" t="inlineStr">
         <is>
           <t>Consistência, conformidade e padronização</t>
         </is>
       </c>
       <c r="C11" s="16" t="n"/>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="35" t="inlineStr">
         <is>
           <t>“data needs to be consistent, complete, and accurate.”, “If this doesn't happen, the entire result from your ML pipeline may be compromised.”, “Conformity is important for the very construction of pipelines, since your data needs to be standardized to be fed into your ML system.”, “Regarding reliability and traceability, the former relates to consistency, which is essential in ML systems.”, “The latter is super important for running tests with older data, performing debugging, or even rollback processes.”</t>
         </is>
       </c>
-      <c r="E11" s="18" t="inlineStr">
+      <c r="E11" s="37" t="inlineStr">
         <is>
           <t>For the development of correct and effective ML systems, data needs to be consistent, complete, and accurate. If this doesn't happen, the entire result from your ML pipeline may be compromised. Conformity is important for the very construction of pipelines, since your data needs to be standardized to be fed into your ML system. Regarding reliability and traceability, the former relates to consistency, which is essential in ML systems, while the latter is super important for running tests with older data, performing debugging, or even rollback processes.</t>
         </is>
@@ -829,23 +829,23 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="35" t="inlineStr">
         <is>
           <t>HIERARQUIZAÇÃO E RELATIVIZAÇÃO DA IMPORTÂNCIA</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B12" s="35" t="inlineStr">
         <is>
           <t>Diferença entre "importante" e "necessário"</t>
         </is>
       </c>
       <c r="C12" s="16" t="n"/>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="35" t="inlineStr">
         <is>
           <t>“there's a difference between something being important and being necessary for a project, especially when it's a pilot project.”, “Often, these two aspects conflict because the importance of certain elements is limited by the urgency of the terms, preventing them from coexisting properly.”</t>
         </is>
       </c>
-      <c r="E12" s="18" t="inlineStr">
+      <c r="E12" s="37" t="inlineStr">
         <is>
           <t>I can imagine several scenarios where all these words are extremely important in some way. However, I believe there's a difference between something being important and being necessary for a project, especially when it's a pilot project. Often, these two aspects conflict because the importance of certain elements is limited by the urgency of the terms, preventing them from coexisting properly.</t>
         </is>
@@ -857,23 +857,23 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="35" t="inlineStr">
         <is>
           <t>HIERARQUIZAÇÃO E RELATIVIZAÇÃO DA IMPORTÂNCIA</t>
         </is>
       </c>
-      <c r="B13" s="15" t="inlineStr">
+      <c r="B13" s="35" t="inlineStr">
         <is>
           <t>Critérios relevantes mas não impeditivos</t>
         </is>
       </c>
       <c r="C13" s="16" t="n"/>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="35" t="inlineStr">
         <is>
           <t>These are relevant criteria, but they do not create impediments.</t>
         </is>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E13" s="36" t="inlineStr">
         <is>
           <t>These are relevant criteria, but they do not create impediments.</t>
         </is>
@@ -885,23 +885,23 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="35" t="inlineStr">
         <is>
           <t>QUALIDADE DOS DADOS COMO FUNDAMENTO INEGOCIÁVEL</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B14" s="35" t="inlineStr">
         <is>
           <t>Impacto positivo no desenvolvimento de sistemas de ML</t>
         </is>
       </c>
       <c r="C14" s="16" t="n"/>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="35" t="inlineStr">
         <is>
           <t>“More current, accurate, and consistent data that reflects the real-world scenario tend to yield better results in the model analysis phase, particularly regarding accuracy metrics.”</t>
         </is>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E14" s="36" t="inlineStr">
         <is>
           <t>More current, accurate, and consistent data that reflects the real-world scenario tend to yield better results in the model analysis phase, particularly regarding accuracy metrics.</t>
         </is>
@@ -913,23 +913,23 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="35" t="inlineStr">
         <is>
           <t>CONSEQUÊNCIAS DA NEGLIGÊNCIA DA QUALIDADE</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B15" s="35" t="inlineStr">
         <is>
           <t>Resultados enganosos ou modelos não-confiáveis</t>
         </is>
       </c>
       <c r="C15" s="16" t="n"/>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="35" t="inlineStr">
         <is>
           <t>“the models created may not reflect the intended objective of the developer/researcher.”, “Or, in worse cases, they may lead to results that may seem promising, but which, upon deeper analysis, may be related to data that is not properly cleaned and accurate.”</t>
         </is>
       </c>
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="37" t="inlineStr">
         <is>
           <t>Given the neglect of these points raised, the models created may not reflect the intended objective of the developer/researcher. Or, in worse cases, they may lead to results that may seem promising, but which, upon deeper analysis, may be related to data that is not properly cleaned and accurate.</t>
         </is>
@@ -941,23 +941,23 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="35" t="inlineStr">
         <is>
           <t>QUALIDADE DOS DADOS COMO FUNDAMENTO INEGOCIÁVEL</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B16" s="35" t="inlineStr">
         <is>
           <t>Caráter não-negociável da qualidade desde o início</t>
         </is>
       </c>
       <c r="C16" s="16" t="n"/>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="D16" s="35" t="inlineStr">
         <is>
           <t>If the data does not have most of these attributes, any result from any ML model will not be reliable.</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E16" s="36" t="inlineStr">
         <is>
           <t>If the data does not have most of these attributes, any result from any ML model will not be reliable.</t>
         </is>
@@ -969,23 +969,23 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
+      <c r="B17" s="35" t="inlineStr">
         <is>
           <t>Confiabilidade e significado dos dados</t>
         </is>
       </c>
       <c r="C17" s="16" t="n"/>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="D17" s="35" t="inlineStr">
         <is>
           <t>"that data must be reliable and meaningful, as this is fundamental for the system to function correctly when put into production.”, “To make decisions based on this data, the information must be accurate and consistent.”</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="37" t="inlineStr">
         <is>
           <t>I believe that data must be reliable and meaningful, as this is fundamental for the system to function correctly when put into production. To make decisions based on this data, the information must be accurate and consistent.</t>
         </is>
@@ -997,24 +997,24 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B18" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">Atualidade, disponibilidade e não-ambiguidade
 </t>
         </is>
       </c>
       <c r="C18" s="16" t="n"/>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="35" t="inlineStr">
         <is>
           <t>“The most fundamental thing is that the data needs to be unambiguous because decision-making needs to be assertive.”, “Taking a critical action, such as blocking a 5-star customer's card, is terrible.”, “Data needs to be always available, consistent, and up-to-date.”, “I see a strong correlation between consistency and timeliness.”, “For example, a customer can become delinquent at any time.”, “Up-to-date data is essential, especially for startups.”</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E18" s="36" t="inlineStr">
         <is>
           <t>The most fundamental thing is that the data needs to be unambiguous because decision-making needs to be assertive. Taking a critical action, such as blocking a 5-star customer's card, is terrible. Data needs to be always available, consistent, and up-to-date. I see a strong correlation between consistency and timeliness. For example, a customer can become delinquent at any time. Up-to-date data is essential, especially for startups.</t>
         </is>
@@ -1026,23 +1026,23 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B19" s="35" t="inlineStr">
         <is>
           <t>Precisão como atributo fundamental</t>
         </is>
       </c>
       <c r="C19" s="16" t="n"/>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="D19" s="35" t="inlineStr">
         <is>
           <t>“Precision is important because imprecise data would cause learning and prediction errors in the models that learn from that data.”, “Completeness is important because in real life the model used might simply not be able to predict an observation correctly because the training data used for that model lacks sufficient examples of that data type.”</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E19" s="37" t="inlineStr">
         <is>
           <t>Precision is important because imprecise data would cause learning and prediction errors in the models that learn from that data. Completeness is important because in real life the model used might simply not be able to predict an observation correctly because the training data used for that model lacks sufficient examples of that data type.</t>
         </is>
@@ -1054,23 +1054,23 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>HIERARQUIZAÇÃO E RELATIVIZAÇÃO DA IMPORTÂNCIA</t>
         </is>
       </c>
-      <c r="B20" s="15" t="inlineStr">
+      <c r="B20" s="35" t="inlineStr">
         <is>
           <t>Importância universal mas modulada</t>
         </is>
       </c>
       <c r="C20" s="16" t="n"/>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="D20" s="35" t="inlineStr">
         <is>
           <t>all of these characteristics are important and need to be taken into account for industrial use. At some level.</t>
         </is>
       </c>
-      <c r="E20" s="18" t="inlineStr">
+      <c r="E20" s="37" t="inlineStr">
         <is>
           <t>I believe that all of these characteristics are important and need to be taken into account for industrial use. At some level.</t>
         </is>
@@ -1082,23 +1082,23 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="35" t="inlineStr">
         <is>
           <t>HIERARQUIZAÇÃO E RELATIVIZAÇÃO DA IMPORTÂNCIA</t>
         </is>
       </c>
-      <c r="B21" s="15" t="inlineStr">
+      <c r="B21" s="35" t="inlineStr">
         <is>
           <t>Critérios relevantes mas não impeditivos</t>
         </is>
       </c>
       <c r="C21" s="16" t="n"/>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="D21" s="35" t="inlineStr">
         <is>
           <t>“Items marked as important do not necessarily mean that the models will perform worse.”, “It is still possible to extract good metrics from a database that includes items marked as Very important.”</t>
         </is>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="E21" s="36" t="inlineStr">
         <is>
           <t>Items marked as important do not necessarily mean that the models will perform worse. It is still possible to extract good metrics from a database that includes items marked as Very important.</t>
         </is>
@@ -1110,23 +1110,23 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B22" s="35" t="inlineStr">
         <is>
           <t>Completude como atributo crítico</t>
         </is>
       </c>
       <c r="C22" s="16" t="n"/>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="D22" s="35" t="inlineStr">
         <is>
           <t>Completeness because incomplete data can minimize usefulness of the ML system derived.</t>
         </is>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E22" s="36" t="inlineStr">
         <is>
           <t>Completeness because incomplete data can minimize usefulness of the ML system derived.</t>
         </is>
@@ -1138,23 +1138,23 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="35" t="inlineStr">
         <is>
           <t>QUALIDADE DOS DADOS COMO FUNDAMENTO INEGOCIÁVEL</t>
         </is>
       </c>
-      <c r="B23" s="15" t="inlineStr">
+      <c r="B23" s="35" t="inlineStr">
         <is>
           <t>Princípio "Garbage In, Garbage Out"</t>
         </is>
       </c>
       <c r="C23" s="16" t="n"/>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="D23" s="35" t="inlineStr">
         <is>
           <t>Because wrong data means wrong results</t>
         </is>
       </c>
-      <c r="E23" s="17" t="inlineStr">
+      <c r="E23" s="36" t="inlineStr">
         <is>
           <t>Because wrong data means wrong results</t>
         </is>
@@ -1166,23 +1166,23 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B24" s="35" t="inlineStr">
         <is>
           <t>Completude como atributo crítico</t>
         </is>
       </c>
       <c r="C24" s="16" t="n"/>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D24" s="35" t="inlineStr">
         <is>
           <t>incompleteness of data may significantly bias the model</t>
         </is>
       </c>
-      <c r="E24" s="17" t="inlineStr">
+      <c r="E24" s="36" t="inlineStr">
         <is>
           <t>incompleteness of data may significantly bias the model. Highly depend  on the project.</t>
         </is>
@@ -1194,24 +1194,24 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="35" t="inlineStr">
         <is>
           <t>ATRIBUTOS TÉCNICOS DA QUALIDADE DOS DADOS</t>
         </is>
       </c>
-      <c r="B25" s="15" t="inlineStr">
+      <c r="B25" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">Rastreabilidade e reprodutibilidade
 </t>
         </is>
       </c>
       <c r="C25" s="16" t="n"/>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="D25" s="35" t="inlineStr">
         <is>
           <t>“I ranked them as important as they are needed for the reproducibility of the results, which is important to have cumulative knowledge.”</t>
         </is>
       </c>
-      <c r="E25" s="18" t="inlineStr">
+      <c r="E25" s="37" t="inlineStr">
         <is>
           <t>you expalined acc. but in rating scale you ask for prec.
 i ranked them as important as they are needed for the reproducibility of the results, whcih is important to have cumulative knowlede.</t>
@@ -1224,23 +1224,23 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="35" t="inlineStr">
         <is>
           <t>Especificidade de domínio</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B26" s="35" t="inlineStr">
         <is>
           <t>Especificidade de domínio</t>
         </is>
       </c>
       <c r="C26" s="16" t="n"/>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="D26" s="35" t="inlineStr">
         <is>
           <t>Industrial engineering consider things differently</t>
         </is>
       </c>
-      <c r="E26" s="17" t="inlineStr">
+      <c r="E26" s="36" t="inlineStr">
         <is>
           <t>Industrial engineering consider things differently</t>
         </is>

</xml_diff>